<commit_message>
Stage 8 review fixes: E-009
</commit_message>
<xml_diff>
--- a/output/archive/WestravelleData/Methods/CU19/WA-2023-136/Results/Approved/CU19_PULLS_AND_SUITABILITY_RESULTS_Rev03.xlsx
+++ b/output/archive/WestravelleData/Methods/CU19/WA-2023-136/Results/Approved/CU19_PULLS_AND_SUITABILITY_RESULTS_Rev03.xlsx
@@ -31,6 +31,10 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="00000000"/>
     </font>
     <font>
@@ -44,10 +48,6 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -80,10 +80,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -460,194 +460,201 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>WA/2023/136 CU19 column-equivalence results</t>
+          <t>Westravelle Analytical Ltd, a Tarnovell company</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>WA/2023/136 CU19 column-equivalence results</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>WA/2023/136</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>LIMS</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>WST-23-004243</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Culdrevane Pharma</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Lead</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Alice Penrose</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Method owner</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Saira Mahmood</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Sequence owner</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Leon Wu</t>
         </is>
       </c>
     </row>
-    <row r="8"/>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="9"/>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Milestone</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Quote accepted</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Quote</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>28/04/2023</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Start of column runs</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>18/05/2023</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Interim data review</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>14/06/2023</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Completion</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>12/07/2023</t>
         </is>
       </c>
     </row>
-    <row r="14"/>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="15"/>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Routine method</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Unchanged; alternate column specified in the method</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Qualified backup for routine release; implementation details remain in the controlled method.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Overall outcome</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Alternate column reproduces required separation of all specified peak pairs</t>
-        </is>
-      </c>
-    </row>
-    <row r="18"/>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Alternate column reproduced the required separation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>Reviewed by</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>Saira Mahmood</t>
         </is>
       </c>
-      <c r="C19" s="2" t="n"/>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="C20" s="3" t="n"/>
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>Checked 12/07/2023</t>
         </is>
@@ -668,7 +675,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -681,202 +688,69 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Column-equivalence sequence: system suitability per column</t>
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Column-equivalence sequence records</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Same mobile phase batch, same sample solutions, same instrument methods. Column serial numbers and lot numbers are recorded on the batch card.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Source record</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Original and alternate column identities</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Refer to the batch card.</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Column</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Role</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Injections</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Rs critical pair</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Tailing (main peak)</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Plates (main peak)</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Outcome</t>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Separation evidence</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Refer to the column-equivalence chromatograms and sequence sheets.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Original column</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Reference</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>6 replicates</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Met</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Met</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Met</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Accepted</t>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>System suitability</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Refer to the sequence-specific acceptance checks.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Alternate column</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Candidate backup</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>6 replicates</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Met</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Met</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Met</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Accepted</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Original column, after 40 injections</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Ageing check</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>3 replicates</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Met</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Met</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Met</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Accepted</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Alternate column, after 40 injections</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Ageing check</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>3 replicates</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Met</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Met</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Met</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>Accepted</t>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Disposition</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Alternate column qualified as a backup for routine release.</t>
         </is>
       </c>
     </row>
@@ -904,154 +778,154 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>HPLC method qualification: summary on the alternate column</t>
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>HPLC method qualification: summary</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Parameters repeated on the alternate column only. Acceptance limits as stated in the transfer protocol.</t>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Qualification parameters are summarised below; column-specific sequence details remain in the transfer records. Acceptance limits as stated in the transfer protocol.</t>
         </is>
       </c>
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Parameter</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Acceptance</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Linearity (r²)</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B5" s="3" t="n">
         <v>0.9995000000000001</v>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>≥0.999</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Range (% nominal)</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>50-150</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>80-120 minimum</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Accuracy 80% (% recovery)</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B7" s="3" t="n">
         <v>100.2</v>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>98.0-102.0</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Accuracy 100% (% recovery)</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n">
+      <c r="B8" s="3" t="n">
         <v>100.2</v>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>98.0-102.0</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Accuracy 120% (% recovery)</t>
         </is>
       </c>
-      <c r="B9" s="2" t="n">
+      <c r="B9" s="3" t="n">
         <v>101.4</v>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>98.0-102.0</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Repeatability (%RSD, n=6)</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n">
+      <c r="B10" s="3" t="n">
         <v>0.28</v>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>≤2.0</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Intermediate precision (%RSD)</t>
         </is>
       </c>
-      <c r="B11" s="2" t="n">
+      <c r="B11" s="3" t="n">
         <v>1.13</v>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>≤2.0</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>LOQ (% of nominal)</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n">
+      <c r="B12" s="3" t="n">
         <v>0.03</v>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>≤0.05</t>
         </is>
@@ -1072,7 +946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -1082,119 +956,81 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>Deviation and sign-off record</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Transfer disposition and review record</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Date</t>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Record</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Retention time drift on the alternate column in the first sequence, memo filed, resolved by longer equilibration</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Damien Grant</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>01/06/2023</t>
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Column-equivalence conclusion</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Alternate column reproduced the required separation.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Column-equivalence conclusion</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Saira Mahmood</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Approved</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Routine release backup</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Qualified; refer to the controlled transfer report and method.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Interim review</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>14/06/2023</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Completion</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>12/07/2023</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Backup column listed in the routine method</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Alice Penrose</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Approved</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>12/07/2023</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Final results and this workbook</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Leon Wu</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Issued Rev03</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>12/07/2023</t>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Deviations and repeats</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Refer to the original sequence sheets; no additional runs are tabulated here.</t>
         </is>
       </c>
     </row>

</xml_diff>